<commit_message>
Add professional button images with menu navigation
- Professional gradient buttons with shadow text
- Main Menu buttons: 500HR, Cust Property, Exchange, Quote Tracker, PO Tracking, Infor XA, Quick Reference
- Action buttons: Generate PDF, Send Email, Clear Form, Menu, Update, etc.
- All buttons embedded in workbook at proper positions
- No overlapping, clean layout
</commit_message>
<xml_diff>
--- a/QAA_Quote_System_v14.xlsx
+++ b/QAA_Quote_System_v14.xlsx
@@ -202,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -243,11 +243,137 @@
         <color rgb="001B365D"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E0E0E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B365D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B365D"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B365D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001B365D"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B365D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B365D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E0E0E0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E0E0E0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E0E0E0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -359,6 +485,14 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,6 +593,501 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1714500" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="361950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -824,21 +1453,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>[ Go500HR ]</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>[ GoCustProp ]</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>[ GoExchange ]</t>
-        </is>
-      </c>
+      <c r="B10" s="7" t="inlineStr"/>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
@@ -891,6 +1508,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="17">
       <c r="B17" s="6" t="inlineStr">
         <is>
@@ -907,6 +1525,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1305,6 +1924,13 @@
           <t>500HR MAGNETO INSPECTION SERVICE QUOTE</t>
         </is>
       </c>
+      <c r="C2" s="57" t="n"/>
+      <c r="D2" s="57" t="n"/>
+      <c r="E2" s="57" t="n"/>
+      <c r="F2" s="57" t="n"/>
+      <c r="G2" s="57" t="n"/>
+      <c r="H2" s="57" t="n"/>
+      <c r="I2" s="58" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="12" t="inlineStr">
@@ -1350,6 +1976,7 @@
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr"/>
+      <c r="G5" s="58" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
@@ -1358,6 +1985,8 @@
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="57" t="n"/>
+      <c r="E6" s="58" t="n"/>
       <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Approval?</t>
@@ -1915,6 +2544,7 @@
         <f>I26+I27+D25</f>
         <v/>
       </c>
+      <c r="I28" s="59" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="4" t="inlineStr">
@@ -1925,8 +2555,24 @@
     </row>
     <row r="31">
       <c r="B31" s="14" t="inlineStr"/>
-    </row>
-    <row r="32"/>
+      <c r="C31" s="60" t="n"/>
+      <c r="D31" s="60" t="n"/>
+      <c r="E31" s="60" t="n"/>
+      <c r="F31" s="60" t="n"/>
+      <c r="G31" s="60" t="n"/>
+      <c r="H31" s="60" t="n"/>
+      <c r="I31" s="61" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="62" t="n"/>
+      <c r="C32" s="63" t="n"/>
+      <c r="D32" s="63" t="n"/>
+      <c r="E32" s="63" t="n"/>
+      <c r="F32" s="63" t="n"/>
+      <c r="G32" s="63" t="n"/>
+      <c r="H32" s="63" t="n"/>
+      <c r="I32" s="64" t="n"/>
+    </row>
     <row r="34">
       <c r="B34" s="6" t="inlineStr">
         <is>
@@ -1935,33 +2581,17 @@
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>[ GENERATE PDF ]</t>
-        </is>
-      </c>
-      <c r="D36" s="27" t="inlineStr">
-        <is>
-          <t>[ SEND EMAIL ]</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="inlineStr">
-        <is>
-          <t>[ CLEAR FORM ]</t>
-        </is>
-      </c>
-      <c r="H36" s="27" t="inlineStr">
-        <is>
-          <t>[ ← MENU ]</t>
-        </is>
-      </c>
+      <c r="B36" s="27" t="inlineStr"/>
+      <c r="D36" s="27" t="inlineStr"/>
+      <c r="F36" s="27" t="inlineStr"/>
+      <c r="H36" s="27" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B34:I34"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B34:I34"/>
     <mergeCell ref="F28:G28"/>
     <mergeCell ref="H28:I28"/>
     <mergeCell ref="B31:I32"/>
@@ -1974,6 +2604,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2010,6 +2641,12 @@
           <t>CUSTOMER PROPERTY OVERHAUL QUOTE</t>
         </is>
       </c>
+      <c r="C2" s="57" t="n"/>
+      <c r="D2" s="57" t="n"/>
+      <c r="E2" s="57" t="n"/>
+      <c r="F2" s="57" t="n"/>
+      <c r="G2" s="57" t="n"/>
+      <c r="H2" s="58" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
@@ -2051,6 +2688,7 @@
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr"/>
+      <c r="G5" s="58" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
@@ -2059,6 +2697,8 @@
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="57" t="n"/>
+      <c r="E6" s="58" t="n"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Tier:</t>
@@ -2450,8 +3090,20 @@
     </row>
     <row r="31">
       <c r="B31" s="14" t="inlineStr"/>
-    </row>
-    <row r="32"/>
+      <c r="C31" s="60" t="n"/>
+      <c r="D31" s="60" t="n"/>
+      <c r="E31" s="60" t="n"/>
+      <c r="F31" s="60" t="n"/>
+      <c r="G31" s="61" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="62" t="n"/>
+      <c r="C32" s="63" t="n"/>
+      <c r="D32" s="63" t="n"/>
+      <c r="E32" s="63" t="n"/>
+      <c r="F32" s="63" t="n"/>
+      <c r="G32" s="64" t="n"/>
+    </row>
     <row r="34">
       <c r="B34" s="6" t="inlineStr">
         <is>
@@ -2460,26 +3112,10 @@
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="34" t="inlineStr">
-        <is>
-          <t>[ GENERATE PDF ]</t>
-        </is>
-      </c>
-      <c r="D36" s="34" t="inlineStr">
-        <is>
-          <t>[ SEND EMAIL ]</t>
-        </is>
-      </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>[ CLEAR ]</t>
-        </is>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>[ MENU ]</t>
-        </is>
-      </c>
+      <c r="B36" s="34" t="inlineStr"/>
+      <c r="D36" s="34" t="inlineStr"/>
+      <c r="F36" s="34" t="inlineStr"/>
+      <c r="H36" s="34" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2500,6 +3136,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2537,6 +3174,15 @@
           <t>EXCHANGE / INVENTORY SALE QUOTE</t>
         </is>
       </c>
+      <c r="B2" s="57" t="n"/>
+      <c r="C2" s="57" t="n"/>
+      <c r="D2" s="57" t="n"/>
+      <c r="E2" s="57" t="n"/>
+      <c r="F2" s="57" t="n"/>
+      <c r="G2" s="57" t="n"/>
+      <c r="H2" s="57" t="n"/>
+      <c r="I2" s="57" t="n"/>
+      <c r="J2" s="58" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -2571,6 +3217,8 @@
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr"/>
+      <c r="C5" s="57" t="n"/>
+      <c r="D5" s="58" t="n"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Tier:</t>
@@ -3089,8 +3737,28 @@
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr"/>
-    </row>
-    <row r="25"/>
+      <c r="B24" s="60" t="n"/>
+      <c r="C24" s="60" t="n"/>
+      <c r="D24" s="60" t="n"/>
+      <c r="E24" s="60" t="n"/>
+      <c r="F24" s="60" t="n"/>
+      <c r="G24" s="60" t="n"/>
+      <c r="H24" s="60" t="n"/>
+      <c r="I24" s="60" t="n"/>
+      <c r="J24" s="61" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="62" t="n"/>
+      <c r="B25" s="63" t="n"/>
+      <c r="C25" s="63" t="n"/>
+      <c r="D25" s="63" t="n"/>
+      <c r="E25" s="63" t="n"/>
+      <c r="F25" s="63" t="n"/>
+      <c r="G25" s="63" t="n"/>
+      <c r="H25" s="63" t="n"/>
+      <c r="I25" s="63" t="n"/>
+      <c r="J25" s="64" t="n"/>
+    </row>
     <row r="27">
       <c r="A27" s="39" t="inlineStr">
         <is>
@@ -3099,26 +3767,10 @@
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="34" t="inlineStr">
-        <is>
-          <t>[ PDF ]</t>
-        </is>
-      </c>
-      <c r="C29" s="34" t="inlineStr">
-        <is>
-          <t>[ EMAIL ]</t>
-        </is>
-      </c>
-      <c r="E29" s="34" t="inlineStr">
-        <is>
-          <t>[ CLEAR ]</t>
-        </is>
-      </c>
-      <c r="G29" s="34" t="inlineStr">
-        <is>
-          <t>[ MENU ]</t>
-        </is>
-      </c>
+      <c r="A29" s="34" t="inlineStr"/>
+      <c r="C29" s="34" t="inlineStr"/>
+      <c r="E29" s="34" t="inlineStr"/>
+      <c r="G29" s="34" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3140,6 +3792,7 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7349,8 +8002,8 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B44:C44"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B44:C44"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B32:C32"/>

</xml_diff>